<commit_message>
docs(SCRUM-165): add complete source AC traceability
</commit_message>
<xml_diff>
--- a/docs/testing/AbangCebu_Modules_3_4_5_Test_Cases.xlsx
+++ b/docs/testing/AbangCebu_Modules_3_4_5_Test_Cases.xlsx
@@ -11,7 +11,7 @@
     <sheet name="TEST_CASES" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'TEST_CASES'!$A$1:$J$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'TEST_CASES'!$A$1:$J$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -436,6 +436,16 @@
           <t>Planning artifact only: no test execution is represented by this workbook.</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Traceability index</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Refer to the per-case criterion trace and execution gates in TEST_CASES.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -469,7 +479,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Traceable functional, security, integration, and recovery test cases derived from SCRUM-125/126/127 planning artifacts and SCRUM-165 acceptance. Resolve listed product/schema gates before implementation; this workbook does not assert product behavior or execution.</t>
+          <t>Traceable functional, security, integration, and recovery test cases derived from SCRUM-125/126/127 planning artifacts and SCRUM-165 acceptance. Acceptance-criterion-to-case traceability is still under review; this draft does not assert full coverage. Resolve listed product/schema gates before execution; this workbook does not assert product behavior or execution.</t>
         </is>
       </c>
     </row>
@@ -493,7 +503,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DEV-2 delivery</t>
+          <t>Project team</t>
         </is>
       </c>
     </row>
@@ -592,7 +602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1805,7 +1815,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Rows 1-23 in this workbook provide planned cases; attached deliverables are planning artifacts only.</t>
+          <t>Primary behavior/data cases are M3-01..M3-07 and X-01..X-05; explicit Module 3/4/5 source-acceptance review cases are M3-A1..M5-A4. Planning only; no execution evidence.</t>
         </is>
       </c>
     </row>
@@ -1905,12 +1915,612 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Live snapshot captured 2026-10-21. Reconcile if source specs/tickets change.</t>
+          <t>Live source/AC crosswalk is partial; X-05 and M3-A1..M5-A4 are designed to expose unverified criteria rather than claim full acceptance coverage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Module 3 - Landlord listing management</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>M3-A1</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>SCRUM-125 AC1: functional scope traces to SCRUM-62, SCRUM-54/55, and existing map docs without contradiction</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Current Jira source tickets and approved spec/ERD/RLS/map docs available to reviewer</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>1. Trace each Module 3 flow/spec element to its cited source. 2. Check table/status names and map handoffs against ERD and map RPC contract. 3. Record each mismatch or unresolved assumption.</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Every scoped flow element has a source; no unsupported status, field, actor, or map behavior is asserted; unresolved conflicts are explicitly listed.</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>High / Requirements trace / design review</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Document/source review, not runtime behavior evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Module 3 - Landlord listing management</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>M3-A2</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>SCRUM-125 AC2: flowcharts include happy path, invalid input, save/resubmit, ownership/authorization, and admin-review handoff</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Current editable Module 3 .drawio sources and corresponding spec</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>1. Inspect each required path in master/subprocess diagrams. 2. Trace invalid-input and save/resubmit branches to persistence/state. 3. Trace ownership and admin handoff to defined roles.</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>All five required flow elements are represented with clear outcomes and correct boundaries; missing or assumed behavior is reported, not inferred.</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>High / Flow coverage / design review</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Use current source artifacts; no implementation claim.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Module 3 - Landlord listing management</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>M3-A3</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>SCRUM-125 AC3: Draw.io source passes structural validation; PDF/PNG exports are legible and match source</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Final .drawio and corresponding final PDF/PNG exports available</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>1. Run the documented structural validator on each source. 2. Regenerate exports from the exact source. 3. Compare branch labels/content. 4. Visually inspect final PDF and PNG at readable scale.</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Validator passes; both exports represent the same final source, include no clipped/hidden required branches, and are legible. Record exact validator/output artifact.</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>High / Artifact QA / visual check</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Visual check remains an execution gate; XML parsing alone is insufficient.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Module 3 - Landlord listing management</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>M3-A4</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>SCRUM-125 AC4: no duplicate auth/map diagrams; assumptions/questions listed in spec</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Current Module 3 docs and existing auth/map flows/specs</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>1. Compare Module 3 diagrams against existing auth/map diagrams. 2. Check auth/map mechanics remain boundary handoffs. 3. Verify every unresolved assumption/question is listed in the spec.</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>No duplicate auth/map workflow; boundaries point to the existing approved flows; unresolved assumptions/questions are explicit.</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Medium / Scope review / documentation</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Check current canonical docs, not Jira filenames alone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Module 4 - Admin KYC and listing moderation</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>M4-A1</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>SCRUM-126 AC1: KYC/listing decisions map to defined statuses, permitted roles, and persisted audit evidence</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Current Module 4 source spec/diagrams, ERD, RLS matrix and audit contract available</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>1. Trace every approve/reject decision to defined status transition. 2. Verify actor against role matrix. 3. Trace persisted audit evidence to schema; mark missing contracts.</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Each decision has an evidenced status, authorized role, and persisted audit mapping; unresolved/missing contracts remain flagged, not assumed.</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Critical / Requirements + security trace</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>No claim that repository implementation currently meets this design criterion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Module 4 - Admin KYC and listing moderation</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>M4-A2</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>SCRUM-126 AC2: reject reason, failed checks, suspicious submissions, appeals/resubmissions, and unauthorized attempts are modeled</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Current editable Module 4 diagrams/spec and policy decision list</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>1. Inspect reject branches for mandatory reason. 2. Inspect failed/suspicious check handling. 3. Inspect appeals/resubmissions and unauthorized-attempt outcomes. 4. Verify open policy cases are surfaced.</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Each listed path has an explicit outcome and authorization boundary; undefined policy is called out and not turned into implemented behavior.</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Critical / Flow coverage + security</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Appeal/suspicious-review policy decisions may block positive runtime tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Module 4 - Admin KYC and listing moderation</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>M4-A3</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>SCRUM-126 AC3: source passes structural validation; exported PDF/PNG match source and are legible</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Final Module 4 .drawio and PDF/PNG exports available</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>1. Run documented structural validator on each .drawio. 2. Regenerate exports. 3. Compare branches/labels to source. 4. Visually inspect final PDF/PNG.</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Validator passes; exports match the exact final source; decision branches are visible and legible. Save validator and final export references.</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>High / Artifact QA / visual check</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Visual QA not established by a source-only review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Module 4 - Admin KYC and listing moderation</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>M4-A4</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>SCRUM-126 AC4: document no implementation claims and explicitly list unresolved policy choices</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Current Module 4 spec, Jira source and diagrams</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>1. Search spec/diagram text for implementation/deployment assertions. 2. Compare every unresolved policy choice in flow to the assumptions/open-questions section.</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Planning content is clearly identified as design, no unverified implementation is claimed, and unresolved policies are explicitly documented.</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>High / Evidence integrity</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Document review only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Module 5 - Renter favorites, contact and inquiry</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>M5-A1</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>SCRUM-127 AC1: flows define authorized transitions, ownership/privacy, persistence, confirmations, and errors</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Current Module 5 spec/diagrams, ERD and RLS matrix</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>1. Trace each favorite/contact/inquiry transition to its permitted actor. 2. Trace persistence and privacy boundary. 3. Verify success confirmation and failure/error paths.</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Every covered flow has an authorized transition, ownership/privacy and persistence mapping, and explicit confirmation/error outcome; gaps are listed.</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Critical / Requirements + privacy trace</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Do not infer runtime enforcement from diagrams.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Module 5 - Renter favorites, contact and inquiry</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>M5-A2</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>SCRUM-127 AC2: authenticated return restores selected listing and original intent; no open redirect or unauthorized contact disclosure</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Current Module 5 and SCRUM-121 auth-gatekeeper source diagrams/spec</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>1. Trace guest high-intent action through auth and return. 2. Verify listing identity and exact intent are preserved. 3. Check destination is constrained to safe same-origin route. 4. Verify contact authorization gate.</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Original authorized intent resumes for the same listing only; unsafe redirects and contact disclosure to unauthorized users are prevented by the specified boundary.</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Critical / Security + redirect/privacy review</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Design review; browser/auth execution separate and not run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Module 5 - Renter favorites, contact and inquiry</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>M5-A3</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>SCRUM-127 AC3: source passes structural validation; PDF/PNG exports match source and are legible</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Final Module 5 .drawio and PDF/PNG exports available</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>1. Run documented structural validator on each source. 2. Regenerate exports. 3. Compare branches/labels to exact source. 4. Visually inspect final PDF/PNG.</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Validator passes; exports match exact final source; branches and labels are legible and unclipped.</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>High / Artifact QA / visual check</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Visual QA not established by XML/source inspection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Module 5 - Renter favorites, contact and inquiry</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>M5-A4</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>SCRUM-127 AC4: trace to SCRUM-61/121 and ERD/RLS, and document assumptions/policy questions</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Current Module 5 source docs, SCRUM-61/121 and ERD/RLS docs</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>1. Trace each module boundary and data/security element to its cited source. 2. Check no auth/map flow is duplicated. 3. Verify unresolved policy assumptions/questions are listed.</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Traceability is explicit; existing auth/map boundaries are reused; every unresolved policy question is visible and not treated as settled.</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>High / Requirements trace / documentation</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Tests the planning artifact criterion, not application behavior.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J26"/>
+  <autoFilter ref="A1:J38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(SCRUM-165): clarify Jira AC coverage limits
</commit_message>
<xml_diff>
--- a/docs/testing/AbangCebu_Modules_3_4_5_Test_Cases.xlsx
+++ b/docs/testing/AbangCebu_Modules_3_4_5_Test_Cases.xlsx
@@ -479,7 +479,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Traceable functional, security, integration, and recovery test cases derived from SCRUM-125/126/127 planning artifacts and SCRUM-165 acceptance. Acceptance-criterion-to-case traceability is still under review; this draft does not assert full coverage. Resolve listed product/schema gates before execution; this workbook does not assert product behavior or execution.</t>
+          <t>Traceable functional, security, integration, and recovery test cases. Each of the four acceptance criteria in the live Jira descriptions for SCRUM-125/126/127 maps to one or more proposed case IDs. Original binary source attachments and referenced Module 3-5 spec files were not content-reviewed, so full source-spec coverage remains unverified. Resolve listed product/schema gates before execution; this workbook does not assert product behavior or execution.</t>
         </is>
       </c>
     </row>
@@ -1915,7 +1915,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Live source/AC crosswalk is partial; X-05 and M3-A1..M5-A4 are designed to expose unverified criteria rather than claim full acceptance coverage.</t>
+          <t>Each live Jira acceptance criterion is mapped to a case ID; independent reconciliation against original source artifacts remains NOT RUN because their content was unavailable. X-05 and M3-A1..M5-A4 remain planning/QA cases; do not claim full source-spec coverage.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(SCRUM-165): improve workbook print layout
</commit_message>
<xml_diff>
--- a/docs/testing/AbangCebu_Modules_3_4_5_Test_Cases.xlsx
+++ b/docs/testing/AbangCebu_Modules_3_4_5_Test_Cases.xlsx
@@ -1,17 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="TEST DEFINITION" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="TEST_CASES" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRINT VIEW" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEST DEFINITION" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEST_CASES" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'TEST_CASES'!$A$1:$J$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PRINT VIEW'!$A$4:$E$41</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'PRINT VIEW'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'PRINT VIEW'!$A$1:$E$41</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'TEST DEFINITION'!$1:$2</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'TEST DEFINITION'!$A$1:$C$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'TEST_CASES'!$A$1:$J$38</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'TEST_CASES'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'TEST_CASES'!$A$1:$J$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,16 +36,92 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Aptos Display"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <i val="1"/>
+      <color rgb="007F6000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <color rgb="0017365D"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <color rgb="0017365D"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <color rgb="00607080"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <color rgb="00202020"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+      <color rgb="0017365D"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="Aptos"/>
+      <color rgb="00202020"/>
+      <sz val="10.5"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0017365D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3F6FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -45,12 +129,105 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="0017365D"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="medium">
+        <color rgb="0017365D"/>
+      </top>
+    </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00AAB7C4"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="medium">
+        <color rgb="0017365D"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAB7C4"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="00AAB7C4"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAB7C4"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="medium">
+        <color rgb="0017365D"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B8C5D1"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="00AAB7C4"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B8C5D1"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -414,185 +591,1391 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="110" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>AbangCebu AI - Modules 3, 4 and 5 Test Specification</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Planning artifact only: no test execution is represented by this workbook.</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Traceability index</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Refer to the per-case criterion trace and execution gates in TEST_CASES.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Project Name:</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>AbangCebu AI</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Module Name:</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Modules 3, 4 and 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="66" customHeight="1">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Test Description:</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Traceable functional, security, integration, and recovery test cases. Each of the four acceptance criteria in the live Jira descriptions for SCRUM-125/126/127 maps to one or more proposed case IDs. Original binary source attachments and referenced Module 3-5 spec files were not content-reviewed, so full source-spec coverage remains unverified. Resolve listed product/schema gates before execution; this workbook does not assert product behavior or execution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>TYPE OF TEST:</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Functional, integration, security, negative, recovery; design-level test cases</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Test Designed by:</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Project team</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Test Executed by:</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>NOT EXECUTED - planning artifact</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Test Status:</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>NOT RUN</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="48" customHeight="1">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Source tickets:</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>SCRUM-125 (Module 3); SCRUM-126 (Module 4); SCRUM-127 (Module 5); SCRUM-54/55/61/62/63/74/121; docs/database/database-erd.md; docs/security/rls-policies.md; docs/security/rbac-matrix.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="48" customHeight="1">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Open decision note:</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Cases tagged POLICY/SCHEMA GATE require owner-approved policy/schema decisions. Do not interpret them as approved behavior or run them against production/shared data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="42" customHeight="1">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Data boundary:</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Use isolated synthetic accounts and records only. Never include real KYC documents, personal data, credentials, or production data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Plan version:</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>1.0 - 2026-10-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Execution evidence:</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>None. Results and actual executor/date must be recorded by the authorized QA session when executed.</t>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>AbangCebu AI — Modules 3, 4 and 5 Test Cases</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Planning only. All cases remain NOT RUN. Use isolated synthetic data; this workbook does not establish product behavior, QA acceptance, staging validation, or production validation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="8" customHeight="1"/>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Case ID</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Module / section</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Priority / type / gate / status</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Trace, preconditions, steps, expected result, evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="280" customHeight="1">
+      <c r="A5" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>M3-01</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>High / Security + integration / schema and RLS gate
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E5" s="15" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-125: landlord creates and edits only own property and units; SCRUM-54/55/63: schema and owner isolation
+PRECONDITIONS / SYNTHETIC DATA
+Isolated DB; active landlord A, landlord B; synthetic draft and property records; approved schema/RLS contract
+TEST STEPS
+1. Authenticate as landlord A. 2. Create/update a property and associated rental unit. 3. Attempt to read/update landlord B's property by known synthetic ID.
+EXPECTED RESULT
+A's authorized own-record operations persist; B's record is not exposed or modified; unauthorized operation fails closed without existence leakage.
+EVIDENCE / NOTES
+Requires local isolated Supabase/Postgres with approved migrations; no staging or production data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="280" customHeight="1">
+      <c r="A6" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>M3-02</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>High / Functional + security / POLICY-SCHEMA GATE
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E6" s="16" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-125: incomplete draft save precedes submit completeness gates; SCRUM-54: draft state contract is unresolved
+PRECONDITIONS / SYNTHETIC DATA
+Isolated DB; landlord A; approved draft representation and RLS/schema decision
+TEST STEPS
+1. Start a property with incomplete fields and no complete rental unit. 2. Save draft. 3. Reload as landlord A. 4. Query as anon.
+EXPECTED RESULT
+Only if an approved draft contract exists, owner can persist/reload incomplete draft; public role cannot discover/read it. Without the approved draft contract, operation remains blocked and state unchanged.
+EVIDENCE / NOTES
+Do not invent a `draft` enum value; ERD property statuses do not define it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="280" customHeight="1">
+      <c r="A7" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>M3-03</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>High / Functional + integration / owner-defined required-field gate
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-125: submission validates complete property, location, valid unit, ownership and supported media policy
+PRECONDITIONS / SYNTHETIC DATA
+Isolated DB; landlord A; approved fields/media policy; one valid and one invalid synthetic candidate
+TEST STEPS
+1. Submit with missing required property fields. 2. Submit with invalid coordinate range/SRID. 3. Submit without a valid unit. 4. Submit with a fully valid owned listing.
+EXPECTED RESULT
+Invalid submissions return field-specific failures and retain previous state; valid submission reaches pending only under the approved contract; no false success or duplicate review handoff.
+EVIDENCE / NOTES
+Do not invent MIME/size limits or mandatory fields absent approved policy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="280" customHeight="1">
+      <c r="A8" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>M3-04</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>High / Integration + security
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E8" s="16" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-125: approved listing discoverability requires an available unit; SCRUM-143 approved-only search
+PRECONDITIONS / SYNTHETIC DATA
+Isolated DB; approved property with one available unit and one with none; guest role
+TEST STEPS
+1. Search approved property with available unit. 2. Mark the only unit unavailable. 3. Repeat same search. 4. Attempt direct lookup of pending/rejected property.
+EXPECTED RESULT
+Approved + available appears per search contract; unavailable-only is omitted; pending/rejected are never exposed publicly.
+EVIDENCE / NOTES
+Use the verified RPC contract and actual anon caller role once integration is available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="280" customHeight="1">
+      <c r="A9" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>M3-05</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>High / Security + storage integration / storage policy gate
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-125: listing edits/uploads are role- and owner-scoped; private media paths are not public listing fields
+PRECONDITIONS / SYNTHETIC DATA
+Isolated storage/DB only; synthetic landlord A/B; synthetic non-sensitive test image; approved storage policy
+TEST STEPS
+1. Upload/remove/reorder synthetic listing photo as owner. 2. Attempt same actions as landlord B and renter. 3. Inspect public search response for private storage paths.
+EXPECTED RESULT
+Only authorized owner/admin operations succeed per policy; unauthorized attempts fail; public response omits private paths and private KYC media.
+EVIDENCE / NOTES
+Do not use real ID/KYC files. Confirm current storage contract before execution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="280" customHeight="1">
+      <c r="A10" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>M3-06</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>High / Security + transition
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E10" s="16" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-125: moderation outcome locks submitted snapshot; owner cannot approve or alter pending review
+PRECONDITIONS / SYNTHETIC DATA
+Isolated DB; landlord A; pending synthetic property with version; separate admin identity
+TEST STEPS
+1. Submit a valid owned listing. 2. As owner, change review snapshot/status while pending. 3. Attempt owner approval. 4. Compare state and audit metadata.
+EXPECTED RESULT
+Owner cannot mutate submitted review snapshot or self-approve; persisted state remains authoritative and audit history is unchanged on denied actions.
+EVIDENCE / NOTES
+Requires approved listing lifecycle and role policies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="280" customHeight="1">
+      <c r="A11" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>M3-07</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>High / Functional + security / SCHEMA-POLICY GATE
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-125: moderation outcome/rejection reason is consumed from persisted evidence, not inferred
+PRECONDITIONS / SYNTHETIC DATA
+Isolated DB; synthetic approved/rejected outcomes with reviewer/time and rejected reason; unresolved resubmission contract
+TEST STEPS
+1. Present valid persisted approval. 2. Present valid rejection with reason. 3. Present rejection without reason and stale/unknown outcome. 4. Attempt resubmission where schema gate is unresolved.
+EXPECTED RESULT
+Valid outcomes display persisted state; invalid/stale outcomes preserve current state and return to admin correction; unsupported resubmission is blocked with no mutation.
+EVIDENCE / NOTES
+Resubmission must not fabricate rejected-to-pending behavior.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="280" customHeight="1">
+      <c r="A12" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>M4-01</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>M4 — Admin moderation</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>Critical / Security + RLS
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-126: admin-only KYC/listing queue; SCRUM-55/63: privacy and admin authorization
+PRECONDITIONS / SYNTHETIC DATA
+Isolated DB; synthetic admin, landlord, renter, anon; fake placeholder KYC record with no real document bytes
+TEST STEPS
+1. Request KYC/moderation queues as anon, renter, landlord and admin. 2. Request another landlord's KYC state. 3. Check returned fields for document URLs/paths.
+EXPECTED RESULT
+Only authorized admin sees review-queue fields; owner sees only own permitted outcome; guests/renters and unrelated landlords receive no private KYC/moderation data.
+EVIDENCE / NOTES
+Private object content and URLs must not be copied into test evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="280" customHeight="1">
+      <c r="A13" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>M4-02</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>M4 — Admin moderation</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Critical / Functional + security / audit atomicity gate
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-126: KYC decision is verified/rejected with reviewer/time; rejected requires actionable reason
+PRECONDITIONS / SYNTHETIC DATA
+Isolated DB; synthetic pending KYC row; authenticated admin; approved decision/audit contract
+TEST STEPS
+1. Approve valid synthetic submission. 2. Reject a different submission with a nonblank reason. 3. Attempt rejection with blank reason. 4. Attempt decision as non-admin.
+EXPECTED RESULT
+Only authorized decisions persist with reviewer/time and required audit evidence; blank reason and non-admin attempts fail with state unchanged.
+EVIDENCE / NOTES
+Do not create real or reusable credentials; auth identity must be disposable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="280" customHeight="1">
+      <c r="A14" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>M4-03</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>M4 — Admin moderation</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>Critical / Functional + authorization
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-126: listing moderation accepts only pending snapshot and supported transitions
+PRECONDITIONS / SYNTHETIC DATA
+Isolated DB; pending property; admin and landlord synthetic roles; ERD-supported states
+TEST STEPS
+1. Approve pending listing as admin. 2. Reject another pending listing with reason. 3. Attempt decision on stale/non-pending snapshot. 4. Attempt approval as landlord.
+EXPECTED RESULT
+Admin's valid supported decision persists reviewer/time; rejection carries reason; stale/duplicate requests conflict safely; landlord cannot decide or self-approve.
+EVIDENCE / NOTES
+Record and schema contract must be reconciled with current migrations before execution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="280" customHeight="1">
+      <c r="A15" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>M4-04</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>M4 — Admin moderation</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
+        <is>
+          <t>Critical / Security + failure injection / audit contract gate
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-126: audit event and moderation decision are atomic; no KYC content in audit
+PRECONDITIONS / SYNTHETIC DATA
+Isolated DB; synthetic pending listing/KYC; admin; test harness can induce audit-write failure safely
+TEST STEPS
+1. Perform valid decision. 2. Verify one matching audit row. 3. In isolated transaction, induce audit-write failure and retry decision. 4. Inspect audit fields for sensitive content.
+EXPECTED RESULT
+Decision and required audit evidence commit atomically; failed audit leaves decision unmodified; audit retains minimal identifiers/action/reason and never KYC bytes/secrets.
+EVIDENCE / NOTES
+Fault injection must affect disposable local DB only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="280" customHeight="1">
+      <c r="A16" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>M4-05</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="inlineStr">
+        <is>
+          <t>M4 — Admin moderation</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="inlineStr">
+        <is>
+          <t>High / Concurrency + integration / transaction/outbox gate
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-126: failed, repeated, and concurrent review attempts do not double-decide or notify
+PRECONDITIONS / SYNTHETIC DATA
+Isolated DB; pending synthetic listing; two admin sessions; notification sink stub/local fake
+TEST STEPS
+1. Submit same decision twice. 2. Submit approve/reject concurrently from two admins. 3. Simulate notification failure after commit. 4. Retry notification path.
+EXPECTED RESULT
+One authoritative state transition/audit decision; stale conflict or idempotent no-op; notification retry does not duplicate the decision.
+EVIDENCE / NOTES
+Notification behavior is testable only after configured channel/outbox contract exists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="280" customHeight="1">
+      <c r="A17" s="14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>M4-06</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>M4 — Admin moderation</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr">
+        <is>
+          <t>High / Security + policy negative / POLICY GATE
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-126: report/appeal/escalation/suspension actions fail closed pending explicit policy
+PRECONDITIONS / SYNTHETIC DATA
+Isolated DB; synthetic listing; no owner-approved intake/appeal/escalation authority configured
+TEST STEPS
+1. Attempt report intake, appeal, escalation, suspension/unpublish through any available interface. 2. Inspect listing state, visibility, and audit table before/after.
+EXPECTED RESULT
+No implied intake/process or unsupported mutation occurs; state/visibility remain unchanged; no fabricated audit decision; unresolved gate is surfaced.
+EVIDENCE / NOTES
+If product owner approves these policies later, create/add separately approved positive cases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="280" customHeight="1">
+      <c r="A18" s="14" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>M5-01</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>Critical / End-to-end + privacy / auth integration gate
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E18" s="16" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-127: guest browse allowed; private favorites/contact/inquiries denied; SCRUM-121 intent restoration
+PRECONDITIONS / SYNTHETIC DATA
+Isolated app/DB; anon guest; approved listing; no real contact data
+TEST STEPS
+1. Browse approved listing as guest. 2. Start favorite, contact, or inquiry action. 3. Complete login in a separate approved test environment. 4. Return to same listing and verify original action intent only.
+EXPECTED RESULT
+Guest browsing works; high-intent action is deferred; no anonymous persistence or contact disclosure; after authentication, exact safe same-origin intent resumes only for the same authorized listing.
+EVIDENCE / NOTES
+Use disposable identities and synthetic listing; no live email delivery without authorization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="280" customHeight="1">
+      <c r="A19" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>M5-02</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>High / Security + integration / SCHEMA GATE
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-127: favorite uniqueness/idempotent save and owner privacy; schema canonical relation decision
+PRECONDITIONS / SYNTHETIC DATA
+Isolated DB; two synthetic renters; approved available property; verified canonical favorite relation/constraint
+TEST STEPS
+1. Save same property twice as renter A. 2. Query renter A and B favorite lists. 3. Attempt insert for renter B while authenticated as A. 4. Remove as A.
+EXPECTED RESULT
+One renter/property row; duplicate save is idempotent or safely rejected per implemented contract; only owner reads/removes own saved record; cross-user write denied.
+EVIDENCE / NOTES
+ERD names `saved_listings`; SCRUM-121 has alternate `saved_properties`; verify canonical actual schema.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="280" customHeight="1">
+      <c r="A20" s="14" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>M5-03</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
+          <t>High / Functional + privacy / SCHEMA GATE
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E20" s="16" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-127: favorite removal remains possible after listing becomes unavailable; save rechecks eligibility
+PRECONDITIONS / SYNTHETIC DATA
+Isolated DB; renter A saved property that changes approved/available lifecycle; resolved favorite schema
+TEST STEPS
+1. Save while eligible. 2. Make listing unavailable/nonpublic through supported test fixture. 3. Remove existing favorite. 4. Attempt a new save against it.
+EXPECTED RESULT
+Existing private association can be removed without revealing listing details; new save rejects ineligible listing and writes no row.
+EVIDENCE / NOTES
+No mutation of shared listing data; use local synthetic fixture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="280" customHeight="1">
+      <c r="A21" s="14" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>M5-04</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>Critical / Security + privacy / POLICY GATE
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-127: contact reveal is authorized and minimum-data; product eligibility remains open
+PRECONDITIONS / SYNTHETIC DATA
+Isolated DB/API boundary; guest, eligible renter, unrelated user; synthetic contact fields and approved listing
+TEST STEPS
+1. Request contact as guest. 2. Request as authenticated renter without approved eligibility policy. 3. Request under a later approved policy for authorized renter. 4. Inspect success and error/log responses.
+EXPECTED RESULT
+Until contact eligibility policy is approved, withhold details. Once approved, only minimum permitted contact data is returned to authorized renter; errors/logs contain no PII.
+EVIDENCE / NOTES
+No real phone/email or production responses in evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="280" customHeight="1">
+      <c r="A22" s="14" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>M5-05</t>
+        </is>
+      </c>
+      <c r="C22" s="14" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="D22" s="14" t="inlineStr">
+        <is>
+          <t>Critical / Integration + RLS / SCHEMA GATE
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E22" s="16" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-127: inquiry/viewing schema canonical decision; renter ownership and valid listing/unit
+PRECONDITIONS / SYNTHETIC DATA
+Isolated DB; renter A/B, landlord A/B; approved property/unit; resolved inquiry-vs-appointment schema contract
+TEST STEPS
+1. Submit inquiry as renter A for property/unit. 2. Verify landlord derives from property ownership. 3. Read/respond as owning landlord. 4. Attempt reads/replies as unrelated renter/landlord.
+EXPECTED RESULT
+Only supported request fields/statuses persist; landlord is server-derived and correctly routed; only renter and owning landlord can see/respond; unrelated users are denied.
+EVIDENCE / NOTES
+ERD uses `inquiries`; SCRUM-121 references `viewing_appointments`; no equivalence assumed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="280" customHeight="1">
+      <c r="A23" s="14" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>M5-06</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>High / Functional + policy / POLICY GATE
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-127: inquiry is not a confirmed appointment without landlord approval; scheduling semantics are open
+PRECONDITIONS / SYNTHETIC DATA
+Isolated DB/API; approved unit; renter and landlord identities; no owner-approved scheduling policy
+TEST STEPS
+1. Submit viewing request with allowed fields. 2. Inspect renter response, landlord inbox, and persisted status. 3. Attempt to label request confirmed without landlord action.
+EXPECTED RESULT
+Request acknowledgement is distinct from confirmed appointment; no unapproved appointment or unsupported status is created; confirmation only follows approved landlord scheduling workflow.
+EVIDENCE / NOTES
+Timezone, slot, reschedule/cancel, and response SLA require owner decision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="280" customHeight="1">
+      <c r="A24" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>M5-07</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>High / Validation + resilience / POLICY GATE
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E24" s="16" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-127: safe form validation, abuse controls, duplicate prevention and notification reliability require defined policy
+PRECONDITIONS / SYNTHETIC DATA
+Isolated DB; synthetic renters; local-only notification sink; approved message/rate/idempotency contract
+TEST STEPS
+1. Submit invalid/oversized/missing fields. 2. Repeat same request under approved idempotency policy. 3. Simulate notification failure and retry. 4. Inspect logs for secrets/PII.
+EXPECTED RESULT
+Invalid/unverifiable input does not persist; duplicate behavior follows approved idempotency contract; notification retry cannot duplicate inquiry; no secrets or unnecessary PII logged.
+EVIDENCE / NOTES
+Do not invent message limits, quotas, retention, or notification channel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="280" customHeight="1">
+      <c r="A25" s="14" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>X-01</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>Cross-module traceability and integration</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr">
+        <is>
+          <t>Critical / Integration + E2E / all dependencies
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E25" s="15" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-125/126/127: Module 3 pending handoff -&gt; Module 4 decision -&gt; Module 5 approved discovery/engagement; ERD/RLS consistency
+PRECONDITIONS / SYNTHETIC DATA
+Isolated disposable Supabase/Postgres with candidate migrations; synthetic landlord/admin/renter records; all schema decisions approved
+TEST STEPS
+1. Apply migrations on disposable DB. 2. Create listing and valid unit as landlord. 3. Submit pending. 4. Decide as admin with reason if rejected. 5. Search approved/available only. 6. Favorite/inquire as renter. 7. Verify database and role isolation.
+EXPECTED RESULT
+End-to-end data states align to approved schema; public only sees eligible approved inventory; audit evidence present; favorites/inquiry ownership correct. Each step records its own actual command/output and dataset.
+EVIDENCE / NOTES
+No existing staging or shared DB. Must be rerunnable from fresh isolated state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="280" customHeight="1">
+      <c r="A26" s="14" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>X-02</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>Cross-module traceability and integration</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>High / Recovery + integration
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E26" s="16" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-125/126/127: rollback/retry recovery must preserve last committed state
+PRECONDITIONS / SYNTHETIC DATA
+Disposable DB; injected migration/data-operation failures; synthetic records only
+TEST STEPS
+1. Fail a draft/save/submit operation before commit. 2. Retry after resolving failure. 3. Simulate stale conflict and duplicate request. 4. Inspect final state and audit rows.
+EXPECTED RESULT
+Failed transaction does not partially persist or claim success; retries reconcile current state and produce no duplicate moderation/favorite/inquiry records.
+EVIDENCE / NOTES
+Only inject faults in disposable DB/local stub. No destructive shared reset.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="280" customHeight="1">
+      <c r="A27" s="14" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>X-03</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>Cross-module traceability and integration</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr">
+        <is>
+          <t>High / Traceability QA
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E27" s="15" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-165 acceptance: each Module 3/4/5 requirement maps to at least one case
+PRECONDITIONS / SYNTHETIC DATA
+All acceptance/spec source docs present and approved for this plan
+TEST STEPS
+1. Walk each acceptance bullet and requirement paragraph in SCRUM-125, SCRUM-126 and SCRUM-127. 2. Match to case ID(s). 3. Flag open policy/schema gates. 4. Verify source inventory against traceability index.
+EXPECTED RESULT
+Every ticket acceptance criterion and in-scope module requirement references a case ID; each case identifies source criterion, expected result, data boundary and execution gate.
+EVIDENCE / NOTES
+Primary behavior/data cases are M3-01..M3-07 and X-01..X-05; explicit Module 3/4/5 source-acceptance review cases are M3-A1..M5-A4. Planning only; no execution evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="280" customHeight="1">
+      <c r="A28" s="14" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>X-04</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>Cross-module traceability and integration</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>High / Evidence integrity
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E28" s="16" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-165 acceptance: plan/report separates expected results from executed evidence
+PRECONDITIONS / SYNTHETIC DATA
+Workbook and test plans available to executor
+TEST STEPS
+1. Confirm initial result status is NOT RUN. 2. When QA executes, record actual build/environment, dataset, executor/date, output artifact, pass/fail/block and defect links. 3. Ensure no PASS is entered absent reproducible observed evidence and identified run snapshot.
+EXPECTED RESULT
+Planned expected results remain separate from actual execution record; no PASS is entered absent reproducible observed evidence and identified run snapshot.
+EVIDENCE / NOTES
+QA-owned execution and acceptance remain separate from planning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="280" customHeight="1">
+      <c r="A29" s="14" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>X-05</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>Cross-module traceability and integration</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>High / Traceability QA
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E29" s="15" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-165 acceptance: source-to-case coverage for SCRUM-125, SCRUM-126, SCRUM-127 and all explicit gates
+PRECONDITIONS / SYNTHETIC DATA
+Workbook and live criteria snapshot available
+TEST STEPS
+1. Validate every source criterion against case mapping. 2. Validate each explicit policy/schema gate is tagged. 3. Check no planning case claims a test was run. 4. Cross-check source versions and status with live Jira.
+EXPECTED RESULT
+Mapping covers the acceptance criteria retrieved for SCRUM-125/126/127; all open gates and NOT RUN states are visible; source-snapshot timestamp is stated.
+EVIDENCE / NOTES
+Each live Jira acceptance criterion is mapped to a case ID; independent reconciliation against original source artifacts remains NOT RUN because their content was unavailable. X-05 and M3-A1..M5-A4 remain planning/QA cases; do not claim full source-spec coverage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="280" customHeight="1">
+      <c r="A30" s="14" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>M3-A1</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>High / Requirements trace / design review
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E30" s="16" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-125 AC1: functional scope traces to SCRUM-62, SCRUM-54/55, and existing map docs without contradiction
+PRECONDITIONS / SYNTHETIC DATA
+Current Jira source tickets and approved spec/ERD/RLS/map docs available to reviewer
+TEST STEPS
+1. Trace each Module 3 flow/spec element to its cited source. 2. Check table/status names and map handoffs against ERD and map RPC contract. 3. Record each mismatch or unresolved assumption.
+EXPECTED RESULT
+Every scoped flow element has a source; no unsupported status, field, actor, or map behavior is asserted; unresolved conflicts are explicitly listed.
+EVIDENCE / NOTES
+Document/source review, not runtime behavior evidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="280" customHeight="1">
+      <c r="A31" s="14" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>M3-A2</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="inlineStr">
+        <is>
+          <t>High / Flow coverage / design review
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E31" s="15" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-125 AC2: flowcharts include happy path, invalid input, save/resubmit, ownership/authorization, and admin-review handoff
+PRECONDITIONS / SYNTHETIC DATA
+Current editable Module 3 .drawio sources and corresponding spec
+TEST STEPS
+1. Inspect each required path in master/subprocess diagrams. 2. Trace invalid-input and save/resubmit branches to persistence/state. 3. Trace ownership and admin handoff to defined roles.
+EXPECTED RESULT
+All five required flow elements are represented with clear outcomes and correct boundaries; missing or assumed behavior is reported, not inferred.
+EVIDENCE / NOTES
+Use current source artifacts; no implementation claim.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="280" customHeight="1">
+      <c r="A32" s="14" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>M3-A3</t>
+        </is>
+      </c>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="D32" s="14" t="inlineStr">
+        <is>
+          <t>High / Artifact QA / visual check
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E32" s="16" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-125 AC3: Draw.io source passes structural validation; PDF/PNG exports are legible and match source
+PRECONDITIONS / SYNTHETIC DATA
+Final .drawio and corresponding final PDF/PNG exports available
+TEST STEPS
+1. Run the documented structural validator on each source. 2. Regenerate exports from the exact source. 3. Compare branch labels/content. 4. Visually inspect final PDF and PNG at readable scale.
+EXPECTED RESULT
+Validator passes; both exports represent the same final source, include no clipped/hidden required branches, and are legible. Record exact validator/output artifact.
+EVIDENCE / NOTES
+Visual check remains an execution gate; XML parsing alone is insufficient.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="280" customHeight="1">
+      <c r="A33" s="14" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>M3-A4</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>Medium / Scope review / documentation
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E33" s="15" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-125 AC4: no duplicate auth/map diagrams; assumptions/questions listed in spec
+PRECONDITIONS / SYNTHETIC DATA
+Current Module 3 docs and existing auth/map flows/specs
+TEST STEPS
+1. Compare Module 3 diagrams against existing auth/map diagrams. 2. Check auth/map mechanics remain boundary handoffs. 3. Verify every unresolved assumption/question is listed in the spec.
+EXPECTED RESULT
+No duplicate auth/map workflow; boundaries point to the existing approved flows; unresolved assumptions/questions are explicit.
+EVIDENCE / NOTES
+Check current canonical docs, not Jira filenames alone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="280" customHeight="1">
+      <c r="A34" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>M4-A1</t>
+        </is>
+      </c>
+      <c r="C34" s="14" t="inlineStr">
+        <is>
+          <t>M4 — Admin moderation</t>
+        </is>
+      </c>
+      <c r="D34" s="14" t="inlineStr">
+        <is>
+          <t>Critical / Requirements + security trace
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E34" s="16" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-126 AC1: KYC/listing decisions map to defined statuses, permitted roles, and persisted audit evidence
+PRECONDITIONS / SYNTHETIC DATA
+Current Module 4 source spec/diagrams, ERD, RLS matrix and audit contract available
+TEST STEPS
+1. Trace every approve/reject decision to defined status transition. 2. Verify actor against role matrix. 3. Trace persisted audit evidence to schema; mark missing contracts.
+EXPECTED RESULT
+Each decision has an evidenced status, authorized role, and persisted audit mapping; unresolved/missing contracts remain flagged, not assumed.
+EVIDENCE / NOTES
+No claim that repository implementation currently meets this design criterion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="280" customHeight="1">
+      <c r="A35" s="14" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="14" t="inlineStr">
+        <is>
+          <t>M4-A2</t>
+        </is>
+      </c>
+      <c r="C35" s="14" t="inlineStr">
+        <is>
+          <t>M4 — Admin moderation</t>
+        </is>
+      </c>
+      <c r="D35" s="14" t="inlineStr">
+        <is>
+          <t>Critical / Flow coverage + security
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E35" s="15" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-126 AC2: reject reason, failed checks, suspicious submissions, appeals/resubmissions, and unauthorized attempts are modeled
+PRECONDITIONS / SYNTHETIC DATA
+Current editable Module 4 diagrams/spec and policy decision list
+TEST STEPS
+1. Inspect reject branches for mandatory reason. 2. Inspect failed/suspicious check handling. 3. Inspect appeals/resubmissions and unauthorized-attempt outcomes. 4. Verify open policy cases are surfaced.
+EXPECTED RESULT
+Each listed path has an explicit outcome and authorization boundary; undefined policy is called out and not turned into implemented behavior.
+EVIDENCE / NOTES
+Appeal/suspicious-review policy decisions may block positive runtime tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="280" customHeight="1">
+      <c r="A36" s="14" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t>M4-A3</t>
+        </is>
+      </c>
+      <c r="C36" s="14" t="inlineStr">
+        <is>
+          <t>M4 — Admin moderation</t>
+        </is>
+      </c>
+      <c r="D36" s="14" t="inlineStr">
+        <is>
+          <t>High / Artifact QA / visual check
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E36" s="16" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-126 AC3: source passes structural validation; exported PDF/PNG match source and are legible
+PRECONDITIONS / SYNTHETIC DATA
+Final Module 4 .drawio and PDF/PNG exports available
+TEST STEPS
+1. Run documented structural validator on each .drawio. 2. Regenerate exports. 3. Compare branches/labels to source. 4. Visually inspect final PDF/PNG.
+EXPECTED RESULT
+Validator passes; exports match the exact final source; decision branches are visible and legible. Save validator and final export references.
+EVIDENCE / NOTES
+Visual QA not established by a source-only review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="280" customHeight="1">
+      <c r="A37" s="14" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t>M4-A4</t>
+        </is>
+      </c>
+      <c r="C37" s="14" t="inlineStr">
+        <is>
+          <t>M4 — Admin moderation</t>
+        </is>
+      </c>
+      <c r="D37" s="14" t="inlineStr">
+        <is>
+          <t>High / Evidence integrity
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E37" s="15" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-126 AC4: document no implementation claims and explicitly list unresolved policy choices
+PRECONDITIONS / SYNTHETIC DATA
+Current Module 4 spec, Jira source and diagrams
+TEST STEPS
+1. Search spec/diagram text for implementation/deployment assertions. 2. Compare every unresolved policy choice in flow to the assumptions/open-questions section.
+EXPECTED RESULT
+Planning content is clearly identified as design, no unverified implementation is claimed, and unresolved policies are explicitly documented.
+EVIDENCE / NOTES
+Document review only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="280" customHeight="1">
+      <c r="A38" s="14" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="14" t="inlineStr">
+        <is>
+          <t>M5-A1</t>
+        </is>
+      </c>
+      <c r="C38" s="14" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="D38" s="14" t="inlineStr">
+        <is>
+          <t>Critical / Requirements + privacy trace
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E38" s="16" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-127 AC1: flows define authorized transitions, ownership/privacy, persistence, confirmations, and errors
+PRECONDITIONS / SYNTHETIC DATA
+Current Module 5 spec/diagrams, ERD and RLS matrix
+TEST STEPS
+1. Trace each favorite/contact/inquiry transition to its permitted actor. 2. Trace persistence and privacy boundary. 3. Verify success confirmation and failure/error paths.
+EXPECTED RESULT
+Every covered flow has an authorized transition, ownership/privacy and persistence mapping, and explicit confirmation/error outcome; gaps are listed.
+EVIDENCE / NOTES
+Do not infer runtime enforcement from diagrams.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="280" customHeight="1">
+      <c r="A39" s="14" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>M5-A2</t>
+        </is>
+      </c>
+      <c r="C39" s="14" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="D39" s="14" t="inlineStr">
+        <is>
+          <t>Critical / Security + redirect/privacy review
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E39" s="15" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-127 AC2: authenticated return restores selected listing and original intent; no open redirect or unauthorized contact disclosure
+PRECONDITIONS / SYNTHETIC DATA
+Current Module 5 and SCRUM-121 auth-gatekeeper source diagrams/spec
+TEST STEPS
+1. Trace guest high-intent action through auth and return. 2. Verify listing identity and exact intent are preserved. 3. Check destination is constrained to safe same-origin route. 4. Verify contact authorization gate.
+EXPECTED RESULT
+Original authorized intent resumes for the same listing only; unsafe redirects and contact disclosure to unauthorized users are prevented by the specified boundary.
+EVIDENCE / NOTES
+Design review; browser/auth execution separate and not run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="280" customHeight="1">
+      <c r="A40" s="14" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>M5-A3</t>
+        </is>
+      </c>
+      <c r="C40" s="14" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="inlineStr">
+        <is>
+          <t>High / Artifact QA / visual check
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E40" s="16" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-127 AC3: source passes structural validation; PDF/PNG exports match source and are legible
+PRECONDITIONS / SYNTHETIC DATA
+Final Module 5 .drawio and PDF/PNG exports available
+TEST STEPS
+1. Run documented structural validator on each source. 2. Regenerate exports. 3. Compare branches/labels to exact source. 4. Visually inspect final PDF/PNG.
+EXPECTED RESULT
+Validator passes; exports match exact final source; branches and labels are legible and unclipped.
+EVIDENCE / NOTES
+Visual QA not established by XML/source inspection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="280" customHeight="1">
+      <c r="A41" s="14" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>M5-A4</t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="inlineStr">
+        <is>
+          <t>High / Requirements trace / documentation
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E41" s="15" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-127 AC4: trace to SCRUM-61/121 and ERD/RLS, and document assumptions/policy questions
+PRECONDITIONS / SYNTHETIC DATA
+Current Module 5 source docs, SCRUM-61/121 and ERD/RLS docs
+TEST STEPS
+1. Trace each module boundary and data/security element to its cited source. 2. Check no auth/map flow is duplicated. 3. Verify unresolved policy assumptions/questions are listed.
+EXPECTED RESULT
+Traceability is explicit; existing auth/map boundaries are reused; every unresolved policy question is visible and not treated as settled.
+EVIDENCE / NOTES
+Tests the planning artifact criterion, not application behavior.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <autoFilter ref="A4:E41"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.35" right="0.35" top="0.35" bottom="0.35" header="0.1" footer="0.1"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;8 Planning only • NOT RUN • Page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <rowBreaks count="18" manualBreakCount="18">
+    <brk id="6" min="0" max="16383" man="1"/>
+    <brk id="8" min="0" max="16383" man="1"/>
+    <brk id="10" min="0" max="16383" man="1"/>
+    <brk id="12" min="0" max="16383" man="1"/>
+    <brk id="14" min="0" max="16383" man="1"/>
+    <brk id="16" min="0" max="16383" man="1"/>
+    <brk id="18" min="0" max="16383" man="1"/>
+    <brk id="20" min="0" max="16383" man="1"/>
+    <brk id="22" min="0" max="16383" man="1"/>
+    <brk id="24" min="0" max="16383" man="1"/>
+    <brk id="26" min="0" max="16383" man="1"/>
+    <brk id="28" min="0" max="16383" man="1"/>
+    <brk id="30" min="0" max="16383" man="1"/>
+    <brk id="32" min="0" max="16383" man="1"/>
+    <brk id="34" min="0" max="16383" man="1"/>
+    <brk id="36" min="0" max="16383" man="1"/>
+    <brk id="38" min="0" max="16383" man="1"/>
+    <brk id="40" min="0" max="16383" man="1"/>
+  </rowBreaks>
 </worksheet>
 </file>
 
@@ -600,70 +1983,258 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr autoPageBreaks="0" fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>AbangCebu AI - Modules 3, 4 and 5 Test Specification</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Planning artifact only: no test execution is represented by this workbook.</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Traceability index</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Refer to the per-case criterion trace and execution gates in TEST_CASES.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Project Name:</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>AbangCebu AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Module Name:</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Modules 3, 4 and 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="66" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Test Description:</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Traceable functional, security, integration, and recovery test cases. Each of the four acceptance criteria in the live Jira descriptions for SCRUM-125/126/127 maps to one or more proposed case IDs. Original binary source attachments and referenced Module 3-5 spec files were not content-reviewed, so full source-spec coverage remains unverified. Resolve listed product/schema gates before execution; this workbook does not assert product behavior or execution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>TYPE OF TEST:</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Functional, integration, security, negative, recovery; design-level test cases</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Test Designed by:</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>Project team</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Test Executed by:</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>NOT EXECUTED - planning artifact</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Test Status:</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>Source tickets:</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>SCRUM-125 (Module 3); SCRUM-126 (Module 4); SCRUM-127 (Module 5); SCRUM-54/55/61/62/63/74/121; docs/database/database-erd.md; docs/security/rls-policies.md; docs/security/rbac-matrix.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>Open decision note:</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>Cases tagged POLICY/SCHEMA GATE require owner-approved policy/schema decisions. Do not interpret them as approved behavior or run them against production/shared data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Data boundary:</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>Use isolated synthetic accounts and records only. Never include real KYC documents, personal data, credentials, or production data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>Plan version:</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>1.0 - 2026-10-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>Execution evidence:</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>None. Results and actual executor/date must be recorded by the authorized QA session when executed.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.35" right="0.35" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="5" scale="90" fitToHeight="0" fitToWidth="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="44" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
-    <col width="33" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
-    <col width="45" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Module</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Case ID</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Requirement / Criterion Trace</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Preconditions / Synthetic Data</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Expected Result / Confirmation</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Priority / Type / Gate</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Status / Actual Result</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Evidence / Notes</t>
         </is>
@@ -673,47 +2244,47 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Module 3 - Landlord listing management</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>M3-01</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>SCRUM-125: landlord creates and edits only own property and units; SCRUM-54/55/63: schema and owner isolation</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>Isolated DB; active landlord A, landlord B; synthetic draft and property records; approved schema/RLS contract</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>1. Authenticate as landlord A. 2. Create/update a property and associated rental unit. 3. Attempt to read/update landlord B's property by known synthetic ID.</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>A's authorized own-record operations persist; B's record is not exposed or modified; unauthorized operation fails closed without existence leakage.</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>High / Security + integration / schema and RLS gate</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="1" t="inlineStr">
         <is>
           <t>Requires local isolated Supabase/Postgres with approved migrations; no staging or production data.</t>
         </is>
@@ -723,47 +2294,47 @@
       <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Module 3 - Landlord listing management</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>M3-02</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>SCRUM-125: incomplete draft save precedes submit completeness gates; SCRUM-54: draft state contract is unresolved</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Isolated DB; landlord A; approved draft representation and RLS/schema decision</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>1. Start a property with incomplete fields and no complete rental unit. 2. Save draft. 3. Reload as landlord A. 4. Query as anon.</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="1" t="inlineStr">
         <is>
           <t>Only if an approved draft contract exists, owner can persist/reload incomplete draft; public role cannot discover/read it. Without the approved draft contract, operation remains blocked and state unchanged.</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="1" t="inlineStr">
         <is>
           <t>High / Functional + security / POLICY-SCHEMA GATE</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="1" t="inlineStr">
         <is>
           <t>Do not invent a `draft` enum value; ERD property statuses do not define it.</t>
         </is>
@@ -773,47 +2344,47 @@
       <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Module 3 - Landlord listing management</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>M3-03</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>SCRUM-125: submission validates complete property, location, valid unit, ownership and supported media policy</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>Isolated DB; landlord A; approved fields/media policy; one valid and one invalid synthetic candidate</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>1. Submit with missing required property fields. 2. Submit with invalid coordinate range/SRID. 3. Submit without a valid unit. 4. Submit with a fully valid owned listing.</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="1" t="inlineStr">
         <is>
           <t>Invalid submissions return field-specific failures and retain previous state; valid submission reaches pending only under the approved contract; no false success or duplicate review handoff.</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="1" t="inlineStr">
         <is>
           <t>High / Functional + integration / owner-defined required-field gate</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" s="1" t="inlineStr">
         <is>
           <t>Do not invent MIME/size limits or mandatory fields absent approved policy.</t>
         </is>
@@ -823,47 +2394,47 @@
       <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Module 3 - Landlord listing management</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>M3-04</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>SCRUM-125: approved listing discoverability requires an available unit; SCRUM-143 approved-only search</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>Isolated DB; approved property with one available unit and one with none; guest role</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="1" t="inlineStr">
         <is>
           <t>1. Search approved property with available unit. 2. Mark the only unit unavailable. 3. Repeat same search. 4. Attempt direct lookup of pending/rejected property.</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="1" t="inlineStr">
         <is>
           <t>Approved + available appears per search contract; unavailable-only is omitted; pending/rejected are never exposed publicly.</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="1" t="inlineStr">
         <is>
           <t>High / Integration + security</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J5" s="1" t="inlineStr">
         <is>
           <t>Use the verified RPC contract and actual anon caller role once integration is available.</t>
         </is>
@@ -873,47 +2444,47 @@
       <c r="A6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Module 3 - Landlord listing management</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>M3-05</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>SCRUM-125: listing edits/uploads are role- and owner-scoped; private media paths are not public listing fields</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>Isolated storage/DB only; synthetic landlord A/B; synthetic non-sensitive test image; approved storage policy</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>1. Upload/remove/reorder synthetic listing photo as owner. 2. Attempt same actions as landlord B and renter. 3. Inspect public search response for private storage paths.</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="1" t="inlineStr">
         <is>
           <t>Only authorized owner/admin operations succeed per policy; unauthorized attempts fail; public response omits private paths and private KYC media.</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="1" t="inlineStr">
         <is>
           <t>High / Security + storage integration / storage policy gate</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J6" s="1" t="inlineStr">
         <is>
           <t>Do not use real ID/KYC files. Confirm current storage contract before execution.</t>
         </is>
@@ -923,47 +2494,47 @@
       <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Module 3 - Landlord listing management</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>M3-06</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="1" t="inlineStr">
         <is>
           <t>SCRUM-125: moderation outcome locks submitted snapshot; owner cannot approve or alter pending review</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>Isolated DB; landlord A; pending synthetic property with version; separate admin identity</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="1" t="inlineStr">
         <is>
           <t>1. Submit a valid owned listing. 2. As owner, change review snapshot/status while pending. 3. Attempt owner approval. 4. Compare state and audit metadata.</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="1" t="inlineStr">
         <is>
           <t>Owner cannot mutate submitted review snapshot or self-approve; persisted state remains authoritative and audit history is unchanged on denied actions.</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="1" t="inlineStr">
         <is>
           <t>High / Security + transition</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J7" s="1" t="inlineStr">
         <is>
           <t>Requires approved listing lifecycle and role policies.</t>
         </is>
@@ -973,47 +2544,47 @@
       <c r="A8" t="n">
         <v>7</v>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Module 3 - Landlord listing management</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>M3-07</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="1" t="inlineStr">
         <is>
           <t>SCRUM-125: moderation outcome/rejection reason is consumed from persisted evidence, not inferred</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>Isolated DB; synthetic approved/rejected outcomes with reviewer/time and rejected reason; unresolved resubmission contract</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
         <is>
           <t>1. Present valid persisted approval. 2. Present valid rejection with reason. 3. Present rejection without reason and stale/unknown outcome. 4. Attempt resubmission where schema gate is unresolved.</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="1" t="inlineStr">
         <is>
           <t>Valid outcomes display persisted state; invalid/stale outcomes preserve current state and return to admin correction; unsupported resubmission is blocked with no mutation.</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H8" s="1" t="inlineStr">
         <is>
           <t>High / Functional + security / SCHEMA-POLICY GATE</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I8" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J8" s="1" t="inlineStr">
         <is>
           <t>Resubmission must not fabricate rejected-to-pending behavior.</t>
         </is>
@@ -1023,47 +2594,47 @@
       <c r="A9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Module 4 - Admin KYC and listing moderation</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>M4 — Admin moderation</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>M4-01</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="1" t="inlineStr">
         <is>
           <t>SCRUM-126: admin-only KYC/listing queue; SCRUM-55/63: privacy and admin authorization</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>Isolated DB; synthetic admin, landlord, renter, anon; fake placeholder KYC record with no real document bytes</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="1" t="inlineStr">
         <is>
           <t>1. Request KYC/moderation queues as anon, renter, landlord and admin. 2. Request another landlord's KYC state. 3. Check returned fields for document URLs/paths.</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" s="1" t="inlineStr">
         <is>
           <t>Only authorized admin sees review-queue fields; owner sees only own permitted outcome; guests/renters and unrelated landlords receive no private KYC/moderation data.</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H9" s="1" t="inlineStr">
         <is>
           <t>Critical / Security + RLS</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I9" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J9" s="1" t="inlineStr">
         <is>
           <t>Private object content and URLs must not be copied into test evidence.</t>
         </is>
@@ -1073,47 +2644,47 @@
       <c r="A10" t="n">
         <v>9</v>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Module 4 - Admin KYC and listing moderation</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>M4 — Admin moderation</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>M4-02</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="1" t="inlineStr">
         <is>
           <t>SCRUM-126: KYC decision is verified/rejected with reviewer/time; rejected requires actionable reason</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="1" t="inlineStr">
         <is>
           <t>Isolated DB; synthetic pending KYC row; authenticated admin; approved decision/audit contract</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="1" t="inlineStr">
         <is>
           <t>1. Approve valid synthetic submission. 2. Reject a different submission with a nonblank reason. 3. Attempt rejection with blank reason. 4. Attempt decision as non-admin.</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" s="1" t="inlineStr">
         <is>
           <t>Only authorized decisions persist with reviewer/time and required audit evidence; blank reason and non-admin attempts fail with state unchanged.</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H10" s="1" t="inlineStr">
         <is>
           <t>Critical / Functional + security / audit atomicity gate</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I10" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J10" s="1" t="inlineStr">
         <is>
           <t>Do not create real or reusable credentials; auth identity must be disposable.</t>
         </is>
@@ -1123,47 +2694,47 @@
       <c r="A11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Module 4 - Admin KYC and listing moderation</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>M4 — Admin moderation</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>M4-03</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>SCRUM-126: listing moderation accepts only pending snapshot and supported transitions</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>Isolated DB; pending property; admin and landlord synthetic roles; ERD-supported states</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>1. Approve pending listing as admin. 2. Reject another pending listing with reason. 3. Attempt decision on stale/non-pending snapshot. 4. Attempt approval as landlord.</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" s="1" t="inlineStr">
         <is>
           <t>Admin's valid supported decision persists reviewer/time; rejection carries reason; stale/duplicate requests conflict safely; landlord cannot decide or self-approve.</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H11" s="1" t="inlineStr">
         <is>
           <t>Critical / Functional + authorization</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I11" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J11" s="1" t="inlineStr">
         <is>
           <t>Record and schema contract must be reconciled with current migrations before execution.</t>
         </is>
@@ -1173,47 +2744,47 @@
       <c r="A12" t="n">
         <v>11</v>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Module 4 - Admin KYC and listing moderation</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>M4 — Admin moderation</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>M4-04</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="1" t="inlineStr">
         <is>
           <t>SCRUM-126: audit event and moderation decision are atomic; no KYC content in audit</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="1" t="inlineStr">
         <is>
           <t>Isolated DB; synthetic pending listing/KYC; admin; test harness can induce audit-write failure safely</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="1" t="inlineStr">
         <is>
           <t>1. Perform valid decision. 2. Verify one matching audit row. 3. In isolated transaction, induce audit-write failure and retry decision. 4. Inspect audit fields for sensitive content.</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G12" s="1" t="inlineStr">
         <is>
           <t>Decision and required audit evidence commit atomically; failed audit leaves decision unmodified; audit retains minimal identifiers/action/reason and never KYC bytes/secrets.</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H12" s="1" t="inlineStr">
         <is>
           <t>Critical / Security + failure injection / audit contract gate</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I12" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J12" s="1" t="inlineStr">
         <is>
           <t>Fault injection must affect disposable local DB only.</t>
         </is>
@@ -1223,47 +2794,47 @@
       <c r="A13" t="n">
         <v>12</v>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Module 4 - Admin KYC and listing moderation</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>M4 — Admin moderation</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>M4-05</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
         <is>
           <t>SCRUM-126: failed, repeated, and concurrent review attempts do not double-decide or notify</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>Isolated DB; pending synthetic listing; two admin sessions; notification sink stub/local fake</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="1" t="inlineStr">
         <is>
           <t>1. Submit same decision twice. 2. Submit approve/reject concurrently from two admins. 3. Simulate notification failure after commit. 4. Retry notification path.</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" s="1" t="inlineStr">
         <is>
           <t>One authoritative state transition/audit decision; stale conflict or idempotent no-op; notification retry does not duplicate the decision.</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H13" s="1" t="inlineStr">
         <is>
           <t>High / Concurrency + integration / transaction/outbox gate</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I13" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J13" s="1" t="inlineStr">
         <is>
           <t>Notification behavior is testable only after configured channel/outbox contract exists.</t>
         </is>
@@ -1273,47 +2844,47 @@
       <c r="A14" t="n">
         <v>13</v>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Module 4 - Admin KYC and listing moderation</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>M4 — Admin moderation</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>M4-06</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>SCRUM-126: report/appeal/escalation/suspension actions fail closed pending explicit policy</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>Isolated DB; synthetic listing; no owner-approved intake/appeal/escalation authority configured</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="1" t="inlineStr">
         <is>
           <t>1. Attempt report intake, appeal, escalation, suspension/unpublish through any available interface. 2. Inspect listing state, visibility, and audit table before/after.</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G14" s="1" t="inlineStr">
         <is>
           <t>No implied intake/process or unsupported mutation occurs; state/visibility remain unchanged; no fabricated audit decision; unresolved gate is surfaced.</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H14" s="1" t="inlineStr">
         <is>
           <t>High / Security + policy negative / POLICY GATE</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I14" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J14" s="1" t="inlineStr">
         <is>
           <t>If product owner approves these policies later, create/add separately approved positive cases.</t>
         </is>
@@ -1323,47 +2894,47 @@
       <c r="A15" t="n">
         <v>14</v>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Module 5 - Renter favorites, contact and inquiry</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>M5-01</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>SCRUM-127: guest browse allowed; private favorites/contact/inquiries denied; SCRUM-121 intent restoration</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="1" t="inlineStr">
         <is>
           <t>Isolated app/DB; anon guest; approved listing; no real contact data</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" s="1" t="inlineStr">
         <is>
           <t>1. Browse approved listing as guest. 2. Start favorite, contact, or inquiry action. 3. Complete login in a separate approved test environment. 4. Return to same listing and verify original action intent only.</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G15" s="1" t="inlineStr">
         <is>
           <t>Guest browsing works; high-intent action is deferred; no anonymous persistence or contact disclosure; after authentication, exact safe same-origin intent resumes only for the same authorized listing.</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H15" s="1" t="inlineStr">
         <is>
           <t>Critical / End-to-end + privacy / auth integration gate</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I15" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="J15" s="1" t="inlineStr">
         <is>
           <t>Use disposable identities and synthetic listing; no live email delivery without authorization.</t>
         </is>
@@ -1373,47 +2944,47 @@
       <c r="A16" t="n">
         <v>15</v>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Module 5 - Renter favorites, contact and inquiry</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>M5-02</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>SCRUM-127: favorite uniqueness/idempotent save and owner privacy; schema canonical relation decision</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>Isolated DB; two synthetic renters; approved available property; verified canonical favorite relation/constraint</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F16" s="1" t="inlineStr">
         <is>
           <t>1. Save same property twice as renter A. 2. Query renter A and B favorite lists. 3. Attempt insert for renter B while authenticated as A. 4. Remove as A.</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G16" s="1" t="inlineStr">
         <is>
           <t>One renter/property row; duplicate save is idempotent or safely rejected per implemented contract; only owner reads/removes own saved record; cross-user write denied.</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H16" s="1" t="inlineStr">
         <is>
           <t>High / Security + integration / SCHEMA GATE</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I16" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J16" s="1" t="inlineStr">
         <is>
           <t>ERD names `saved_listings`; SCRUM-121 has alternate `saved_properties`; verify canonical actual schema.</t>
         </is>
@@ -1423,47 +2994,47 @@
       <c r="A17" t="n">
         <v>16</v>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Module 5 - Renter favorites, contact and inquiry</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
         <is>
           <t>M5-03</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="1" t="inlineStr">
         <is>
           <t>SCRUM-127: favorite removal remains possible after listing becomes unavailable; save rechecks eligibility</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="1" t="inlineStr">
         <is>
           <t>Isolated DB; renter A saved property that changes approved/available lifecycle; resolved favorite schema</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="1" t="inlineStr">
         <is>
           <t>1. Save while eligible. 2. Make listing unavailable/nonpublic through supported test fixture. 3. Remove existing favorite. 4. Attempt a new save against it.</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" s="1" t="inlineStr">
         <is>
           <t>Existing private association can be removed without revealing listing details; new save rejects ineligible listing and writes no row.</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="H17" s="1" t="inlineStr">
         <is>
           <t>High / Functional + privacy / SCHEMA GATE</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I17" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="J17" s="1" t="inlineStr">
         <is>
           <t>No mutation of shared listing data; use local synthetic fixture.</t>
         </is>
@@ -1473,47 +3044,47 @@
       <c r="A18" t="n">
         <v>17</v>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Module 5 - Renter favorites, contact and inquiry</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>M5-04</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="1" t="inlineStr">
         <is>
           <t>SCRUM-127: contact reveal is authorized and minimum-data; product eligibility remains open</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>Isolated DB/API boundary; guest, eligible renter, unrelated user; synthetic contact fields and approved listing</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>1. Request contact as guest. 2. Request as authenticated renter without approved eligibility policy. 3. Request under a later approved policy for authorized renter. 4. Inspect success and error/log responses.</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G18" s="1" t="inlineStr">
         <is>
           <t>Until contact eligibility policy is approved, withhold details. Once approved, only minimum permitted contact data is returned to authorized renter; errors/logs contain no PII.</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="H18" s="1" t="inlineStr">
         <is>
           <t>Critical / Security + privacy / POLICY GATE</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="I18" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="J18" s="1" t="inlineStr">
         <is>
           <t>No real phone/email or production responses in evidence.</t>
         </is>
@@ -1523,47 +3094,47 @@
       <c r="A19" t="n">
         <v>18</v>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Module 5 - Renter favorites, contact and inquiry</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
         <is>
           <t>M5-05</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="1" t="inlineStr">
         <is>
           <t>SCRUM-127: inquiry/viewing schema canonical decision; renter ownership and valid listing/unit</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>Isolated DB; renter A/B, landlord A/B; approved property/unit; resolved inquiry-vs-appointment schema contract</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>1. Submit inquiry as renter A for property/unit. 2. Verify landlord derives from property ownership. 3. Read/respond as owning landlord. 4. Attempt reads/replies as unrelated renter/landlord.</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G19" s="1" t="inlineStr">
         <is>
           <t>Only supported request fields/statuses persist; landlord is server-derived and correctly routed; only renter and owning landlord can see/respond; unrelated users are denied.</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="H19" s="1" t="inlineStr">
         <is>
           <t>Critical / Integration + RLS / SCHEMA GATE</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I19" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="J19" s="1" t="inlineStr">
         <is>
           <t>ERD uses `inquiries`; SCRUM-121 references `viewing_appointments`; no equivalence assumed.</t>
         </is>
@@ -1573,47 +3144,47 @@
       <c r="A20" t="n">
         <v>19</v>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Module 5 - Renter favorites, contact and inquiry</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
         <is>
           <t>M5-06</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="1" t="inlineStr">
         <is>
           <t>SCRUM-127: inquiry is not a confirmed appointment without landlord approval; scheduling semantics are open</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>Isolated DB/API; approved unit; renter and landlord identities; no owner-approved scheduling policy</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>1. Submit viewing request with allowed fields. 2. Inspect renter response, landlord inbox, and persisted status. 3. Attempt to label request confirmed without landlord action.</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G20" s="1" t="inlineStr">
         <is>
           <t>Request acknowledgement is distinct from confirmed appointment; no unapproved appointment or unsupported status is created; confirmation only follows approved landlord scheduling workflow.</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H20" s="1" t="inlineStr">
         <is>
           <t>High / Functional + policy / POLICY GATE</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I20" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="J20" s="1" t="inlineStr">
         <is>
           <t>Timezone, slot, reschedule/cancel, and response SLA require owner decision.</t>
         </is>
@@ -1623,47 +3194,47 @@
       <c r="A21" t="n">
         <v>20</v>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Module 5 - Renter favorites, contact and inquiry</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
+      <c r="B21" s="1" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>M5-07</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>SCRUM-127: safe form validation, abuse controls, duplicate prevention and notification reliability require defined policy</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>Isolated DB; synthetic renters; local-only notification sink; approved message/rate/idempotency contract</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>1. Submit invalid/oversized/missing fields. 2. Repeat same request under approved idempotency policy. 3. Simulate notification failure and retry. 4. Inspect logs for secrets/PII.</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G21" s="1" t="inlineStr">
         <is>
           <t>Invalid/unverifiable input does not persist; duplicate behavior follows approved idempotency contract; notification retry cannot duplicate inquiry; no secrets or unnecessary PII logged.</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H21" s="1" t="inlineStr">
         <is>
           <t>High / Validation + resilience / POLICY GATE</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I21" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="J21" s="1" t="inlineStr">
         <is>
           <t>Do not invent message limits, quotas, retention, or notification channel.</t>
         </is>
@@ -1673,47 +3244,47 @@
       <c r="A22" t="n">
         <v>21</v>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>Cross-module traceability and integration</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="1" t="inlineStr">
         <is>
           <t>X-01</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="1" t="inlineStr">
         <is>
           <t>SCRUM-125/126/127: Module 3 pending handoff -&gt; Module 4 decision -&gt; Module 5 approved discovery/engagement; ERD/RLS consistency</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>Isolated disposable Supabase/Postgres with candidate migrations; synthetic landlord/admin/renter records; all schema decisions approved</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t>1. Apply migrations on disposable DB. 2. Create listing and valid unit as landlord. 3. Submit pending. 4. Decide as admin with reason if rejected. 5. Search approved/available only. 6. Favorite/inquire as renter. 7. Verify database and role isolation.</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G22" s="1" t="inlineStr">
         <is>
           <t>End-to-end data states align to approved schema; public only sees eligible approved inventory; audit evidence present; favorites/inquiry ownership correct. Each step records its own actual command/output and dataset.</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="H22" s="1" t="inlineStr">
         <is>
           <t>Critical / Integration + E2E / all dependencies</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="I22" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="J22" s="1" t="inlineStr">
         <is>
           <t>No existing staging or shared DB. Must be rerunnable from fresh isolated state.</t>
         </is>
@@ -1723,47 +3294,47 @@
       <c r="A23" t="n">
         <v>22</v>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>Cross-module traceability and integration</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="1" t="inlineStr">
         <is>
           <t>X-02</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="1" t="inlineStr">
         <is>
           <t>SCRUM-125/126/127: rollback/retry recovery must preserve last committed state</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>Disposable DB; injected migration/data-operation failures; synthetic records only</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F23" s="1" t="inlineStr">
         <is>
           <t>1. Fail a draft/save/submit operation before commit. 2. Retry after resolving failure. 3. Simulate stale conflict and duplicate request. 4. Inspect final state and audit rows.</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G23" s="1" t="inlineStr">
         <is>
           <t>Failed transaction does not partially persist or claim success; retries reconcile current state and produce no duplicate moderation/favorite/inquiry records.</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H23" s="1" t="inlineStr">
         <is>
           <t>High / Recovery + integration</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I23" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="J23" s="1" t="inlineStr">
         <is>
           <t>Only inject faults in disposable DB/local stub. No destructive shared reset.</t>
         </is>
@@ -1773,47 +3344,47 @@
       <c r="A24" t="n">
         <v>23</v>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>Cross-module traceability and integration</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="1" t="inlineStr">
         <is>
           <t>X-03</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="1" t="inlineStr">
         <is>
           <t>SCRUM-165 acceptance: each Module 3/4/5 requirement maps to at least one case</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" s="1" t="inlineStr">
         <is>
           <t>All acceptance/spec source docs present and approved for this plan</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F24" s="1" t="inlineStr">
         <is>
           <t>1. Walk each acceptance bullet and requirement paragraph in SCRUM-125, SCRUM-126 and SCRUM-127. 2. Match to case ID(s). 3. Flag open policy/schema gates. 4. Verify source inventory against traceability index.</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G24" s="1" t="inlineStr">
         <is>
           <t>Every ticket acceptance criterion and in-scope module requirement references a case ID; each case identifies source criterion, expected result, data boundary and execution gate.</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H24" s="1" t="inlineStr">
         <is>
           <t>High / Traceability QA</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="I24" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="J24" s="1" t="inlineStr">
         <is>
           <t>Primary behavior/data cases are M3-01..M3-07 and X-01..X-05; explicit Module 3/4/5 source-acceptance review cases are M3-A1..M5-A4. Planning only; no execution evidence.</t>
         </is>
@@ -1823,47 +3394,47 @@
       <c r="A25" t="n">
         <v>24</v>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="1" t="inlineStr">
         <is>
           <t>Cross-module traceability and integration</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="1" t="inlineStr">
         <is>
           <t>X-04</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="1" t="inlineStr">
         <is>
           <t>SCRUM-165 acceptance: plan/report separates expected results from executed evidence</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="1" t="inlineStr">
         <is>
           <t>Workbook and test plans available to executor</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F25" s="1" t="inlineStr">
         <is>
           <t>1. Confirm initial result status is NOT RUN. 2. When QA executes, record actual build/environment, dataset, executor/date, output artifact, pass/fail/block and defect links. 3. Ensure no PASS is entered absent reproducible observed evidence and identified run snapshot.</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G25" s="1" t="inlineStr">
         <is>
           <t>Planned expected results remain separate from actual execution record; no PASS is entered absent reproducible observed evidence and identified run snapshot.</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H25" s="1" t="inlineStr">
         <is>
           <t>High / Evidence integrity</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="I25" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="J25" s="1" t="inlineStr">
         <is>
           <t>QA-owned execution and acceptance remain separate from planning.</t>
         </is>
@@ -1873,47 +3444,47 @@
       <c r="A26" t="n">
         <v>25</v>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="1" t="inlineStr">
         <is>
           <t>Cross-module traceability and integration</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="1" t="inlineStr">
         <is>
           <t>X-05</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="1" t="inlineStr">
         <is>
           <t>SCRUM-165 acceptance: source-to-case coverage for SCRUM-125, SCRUM-126, SCRUM-127 and all explicit gates</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" s="1" t="inlineStr">
         <is>
           <t>Workbook and live criteria snapshot available</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F26" s="1" t="inlineStr">
         <is>
           <t>1. Validate every source criterion against case mapping. 2. Validate each explicit policy/schema gate is tagged. 3. Check no planning case claims a test was run. 4. Cross-check source versions and status with live Jira.</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G26" s="1" t="inlineStr">
         <is>
           <t>Mapping covers the acceptance criteria retrieved for SCRUM-125/126/127; all open gates and NOT RUN states are visible; source-snapshot timestamp is stated.</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="H26" s="1" t="inlineStr">
         <is>
           <t>High / Traceability QA</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="I26" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="J26" s="1" t="inlineStr">
         <is>
           <t>Each live Jira acceptance criterion is mapped to a case ID; independent reconciliation against original source artifacts remains NOT RUN because their content was unavailable. X-05 and M3-A1..M5-A4 remain planning/QA cases; do not claim full source-spec coverage.</t>
         </is>
@@ -1923,47 +3494,47 @@
       <c r="A27" t="n">
         <v>26</v>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Module 3 - Landlord listing management</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
+      <c r="B27" s="1" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="C27" s="1" t="inlineStr">
         <is>
           <t>M3-A1</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="1" t="inlineStr">
         <is>
           <t>SCRUM-125 AC1: functional scope traces to SCRUM-62, SCRUM-54/55, and existing map docs without contradiction</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" s="1" t="inlineStr">
         <is>
           <t>Current Jira source tickets and approved spec/ERD/RLS/map docs available to reviewer</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F27" s="1" t="inlineStr">
         <is>
           <t>1. Trace each Module 3 flow/spec element to its cited source. 2. Check table/status names and map handoffs against ERD and map RPC contract. 3. Record each mismatch or unresolved assumption.</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" s="1" t="inlineStr">
         <is>
           <t>Every scoped flow element has a source; no unsupported status, field, actor, or map behavior is asserted; unresolved conflicts are explicitly listed.</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="H27" s="1" t="inlineStr">
         <is>
           <t>High / Requirements trace / design review</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="I27" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="J27" s="1" t="inlineStr">
         <is>
           <t>Document/source review, not runtime behavior evidence.</t>
         </is>
@@ -1973,47 +3544,47 @@
       <c r="A28" t="n">
         <v>27</v>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Module 3 - Landlord listing management</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
+      <c r="B28" s="1" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="C28" s="1" t="inlineStr">
         <is>
           <t>M3-A2</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="1" t="inlineStr">
         <is>
           <t>SCRUM-125 AC2: flowcharts include happy path, invalid input, save/resubmit, ownership/authorization, and admin-review handoff</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" s="1" t="inlineStr">
         <is>
           <t>Current editable Module 3 .drawio sources and corresponding spec</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F28" s="1" t="inlineStr">
         <is>
           <t>1. Inspect each required path in master/subprocess diagrams. 2. Trace invalid-input and save/resubmit branches to persistence/state. 3. Trace ownership and admin handoff to defined roles.</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G28" s="1" t="inlineStr">
         <is>
           <t>All five required flow elements are represented with clear outcomes and correct boundaries; missing or assumed behavior is reported, not inferred.</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H28" s="1" t="inlineStr">
         <is>
           <t>High / Flow coverage / design review</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="I28" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="J28" s="1" t="inlineStr">
         <is>
           <t>Use current source artifacts; no implementation claim.</t>
         </is>
@@ -2023,47 +3594,47 @@
       <c r="A29" t="n">
         <v>28</v>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Module 3 - Landlord listing management</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
+      <c r="B29" s="1" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="C29" s="1" t="inlineStr">
         <is>
           <t>M3-A3</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="1" t="inlineStr">
         <is>
           <t>SCRUM-125 AC3: Draw.io source passes structural validation; PDF/PNG exports are legible and match source</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" s="1" t="inlineStr">
         <is>
           <t>Final .drawio and corresponding final PDF/PNG exports available</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F29" s="1" t="inlineStr">
         <is>
           <t>1. Run the documented structural validator on each source. 2. Regenerate exports from the exact source. 3. Compare branch labels/content. 4. Visually inspect final PDF and PNG at readable scale.</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G29" s="1" t="inlineStr">
         <is>
           <t>Validator passes; both exports represent the same final source, include no clipped/hidden required branches, and are legible. Record exact validator/output artifact.</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H29" s="1" t="inlineStr">
         <is>
           <t>High / Artifact QA / visual check</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="I29" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="J29" s="1" t="inlineStr">
         <is>
           <t>Visual check remains an execution gate; XML parsing alone is insufficient.</t>
         </is>
@@ -2073,47 +3644,47 @@
       <c r="A30" t="n">
         <v>29</v>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Module 3 - Landlord listing management</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
+      <c r="B30" s="1" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="C30" s="1" t="inlineStr">
         <is>
           <t>M3-A4</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="1" t="inlineStr">
         <is>
           <t>SCRUM-125 AC4: no duplicate auth/map diagrams; assumptions/questions listed in spec</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E30" s="1" t="inlineStr">
         <is>
           <t>Current Module 3 docs and existing auth/map flows/specs</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F30" s="1" t="inlineStr">
         <is>
           <t>1. Compare Module 3 diagrams against existing auth/map diagrams. 2. Check auth/map mechanics remain boundary handoffs. 3. Verify every unresolved assumption/question is listed in the spec.</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G30" s="1" t="inlineStr">
         <is>
           <t>No duplicate auth/map workflow; boundaries point to the existing approved flows; unresolved assumptions/questions are explicit.</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="H30" s="1" t="inlineStr">
         <is>
           <t>Medium / Scope review / documentation</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="I30" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="J30" s="1" t="inlineStr">
         <is>
           <t>Check current canonical docs, not Jira filenames alone.</t>
         </is>
@@ -2123,47 +3694,47 @@
       <c r="A31" t="n">
         <v>30</v>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Module 4 - Admin KYC and listing moderation</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
+      <c r="B31" s="1" t="inlineStr">
+        <is>
+          <t>M4 — Admin moderation</t>
+        </is>
+      </c>
+      <c r="C31" s="1" t="inlineStr">
         <is>
           <t>M4-A1</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="1" t="inlineStr">
         <is>
           <t>SCRUM-126 AC1: KYC/listing decisions map to defined statuses, permitted roles, and persisted audit evidence</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="1" t="inlineStr">
         <is>
           <t>Current Module 4 source spec/diagrams, ERD, RLS matrix and audit contract available</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F31" s="1" t="inlineStr">
         <is>
           <t>1. Trace every approve/reject decision to defined status transition. 2. Verify actor against role matrix. 3. Trace persisted audit evidence to schema; mark missing contracts.</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G31" s="1" t="inlineStr">
         <is>
           <t>Each decision has an evidenced status, authorized role, and persisted audit mapping; unresolved/missing contracts remain flagged, not assumed.</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="H31" s="1" t="inlineStr">
         <is>
           <t>Critical / Requirements + security trace</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="I31" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="J31" s="1" t="inlineStr">
         <is>
           <t>No claim that repository implementation currently meets this design criterion.</t>
         </is>
@@ -2173,47 +3744,47 @@
       <c r="A32" t="n">
         <v>31</v>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Module 4 - Admin KYC and listing moderation</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
+      <c r="B32" s="1" t="inlineStr">
+        <is>
+          <t>M4 — Admin moderation</t>
+        </is>
+      </c>
+      <c r="C32" s="1" t="inlineStr">
         <is>
           <t>M4-A2</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="1" t="inlineStr">
         <is>
           <t>SCRUM-126 AC2: reject reason, failed checks, suspicious submissions, appeals/resubmissions, and unauthorized attempts are modeled</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="1" t="inlineStr">
         <is>
           <t>Current editable Module 4 diagrams/spec and policy decision list</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" s="1" t="inlineStr">
         <is>
           <t>1. Inspect reject branches for mandatory reason. 2. Inspect failed/suspicious check handling. 3. Inspect appeals/resubmissions and unauthorized-attempt outcomes. 4. Verify open policy cases are surfaced.</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G32" s="1" t="inlineStr">
         <is>
           <t>Each listed path has an explicit outcome and authorization boundary; undefined policy is called out and not turned into implemented behavior.</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="H32" s="1" t="inlineStr">
         <is>
           <t>Critical / Flow coverage + security</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="I32" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="J32" s="1" t="inlineStr">
         <is>
           <t>Appeal/suspicious-review policy decisions may block positive runtime tests.</t>
         </is>
@@ -2223,47 +3794,47 @@
       <c r="A33" t="n">
         <v>32</v>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Module 4 - Admin KYC and listing moderation</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
+      <c r="B33" s="1" t="inlineStr">
+        <is>
+          <t>M4 — Admin moderation</t>
+        </is>
+      </c>
+      <c r="C33" s="1" t="inlineStr">
         <is>
           <t>M4-A3</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="1" t="inlineStr">
         <is>
           <t>SCRUM-126 AC3: source passes structural validation; exported PDF/PNG match source and are legible</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" s="1" t="inlineStr">
         <is>
           <t>Final Module 4 .drawio and PDF/PNG exports available</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F33" s="1" t="inlineStr">
         <is>
           <t>1. Run documented structural validator on each .drawio. 2. Regenerate exports. 3. Compare branches/labels to source. 4. Visually inspect final PDF/PNG.</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="G33" s="1" t="inlineStr">
         <is>
           <t>Validator passes; exports match the exact final source; decision branches are visible and legible. Save validator and final export references.</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="H33" s="1" t="inlineStr">
         <is>
           <t>High / Artifact QA / visual check</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="I33" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="J33" s="1" t="inlineStr">
         <is>
           <t>Visual QA not established by a source-only review.</t>
         </is>
@@ -2273,47 +3844,47 @@
       <c r="A34" t="n">
         <v>33</v>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Module 4 - Admin KYC and listing moderation</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
+      <c r="B34" s="1" t="inlineStr">
+        <is>
+          <t>M4 — Admin moderation</t>
+        </is>
+      </c>
+      <c r="C34" s="1" t="inlineStr">
         <is>
           <t>M4-A4</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="1" t="inlineStr">
         <is>
           <t>SCRUM-126 AC4: document no implementation claims and explicitly list unresolved policy choices</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" s="1" t="inlineStr">
         <is>
           <t>Current Module 4 spec, Jira source and diagrams</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F34" s="1" t="inlineStr">
         <is>
           <t>1. Search spec/diagram text for implementation/deployment assertions. 2. Compare every unresolved policy choice in flow to the assumptions/open-questions section.</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G34" s="1" t="inlineStr">
         <is>
           <t>Planning content is clearly identified as design, no unverified implementation is claimed, and unresolved policies are explicitly documented.</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="H34" s="1" t="inlineStr">
         <is>
           <t>High / Evidence integrity</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="I34" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="J34" s="1" t="inlineStr">
         <is>
           <t>Document review only.</t>
         </is>
@@ -2323,47 +3894,47 @@
       <c r="A35" t="n">
         <v>34</v>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Module 5 - Renter favorites, contact and inquiry</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
+      <c r="B35" s="1" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="C35" s="1" t="inlineStr">
         <is>
           <t>M5-A1</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="1" t="inlineStr">
         <is>
           <t>SCRUM-127 AC1: flows define authorized transitions, ownership/privacy, persistence, confirmations, and errors</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E35" s="1" t="inlineStr">
         <is>
           <t>Current Module 5 spec/diagrams, ERD and RLS matrix</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F35" s="1" t="inlineStr">
         <is>
           <t>1. Trace each favorite/contact/inquiry transition to its permitted actor. 2. Trace persistence and privacy boundary. 3. Verify success confirmation and failure/error paths.</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G35" s="1" t="inlineStr">
         <is>
           <t>Every covered flow has an authorized transition, ownership/privacy and persistence mapping, and explicit confirmation/error outcome; gaps are listed.</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="H35" s="1" t="inlineStr">
         <is>
           <t>Critical / Requirements + privacy trace</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="I35" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="J35" s="1" t="inlineStr">
         <is>
           <t>Do not infer runtime enforcement from diagrams.</t>
         </is>
@@ -2373,47 +3944,47 @@
       <c r="A36" t="n">
         <v>35</v>
       </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Module 5 - Renter favorites, contact and inquiry</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
+      <c r="B36" s="1" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="C36" s="1" t="inlineStr">
         <is>
           <t>M5-A2</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="1" t="inlineStr">
         <is>
           <t>SCRUM-127 AC2: authenticated return restores selected listing and original intent; no open redirect or unauthorized contact disclosure</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E36" s="1" t="inlineStr">
         <is>
           <t>Current Module 5 and SCRUM-121 auth-gatekeeper source diagrams/spec</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F36" s="1" t="inlineStr">
         <is>
           <t>1. Trace guest high-intent action through auth and return. 2. Verify listing identity and exact intent are preserved. 3. Check destination is constrained to safe same-origin route. 4. Verify contact authorization gate.</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G36" s="1" t="inlineStr">
         <is>
           <t>Original authorized intent resumes for the same listing only; unsafe redirects and contact disclosure to unauthorized users are prevented by the specified boundary.</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="H36" s="1" t="inlineStr">
         <is>
           <t>Critical / Security + redirect/privacy review</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="I36" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="J36" s="1" t="inlineStr">
         <is>
           <t>Design review; browser/auth execution separate and not run.</t>
         </is>
@@ -2423,47 +3994,47 @@
       <c r="A37" t="n">
         <v>36</v>
       </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Module 5 - Renter favorites, contact and inquiry</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
+      <c r="B37" s="1" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="C37" s="1" t="inlineStr">
         <is>
           <t>M5-A3</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="1" t="inlineStr">
         <is>
           <t>SCRUM-127 AC3: source passes structural validation; PDF/PNG exports match source and are legible</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E37" s="1" t="inlineStr">
         <is>
           <t>Final Module 5 .drawio and PDF/PNG exports available</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F37" s="1" t="inlineStr">
         <is>
           <t>1. Run documented structural validator on each source. 2. Regenerate exports. 3. Compare branches/labels to exact source. 4. Visually inspect final PDF/PNG.</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G37" s="1" t="inlineStr">
         <is>
           <t>Validator passes; exports match exact final source; branches and labels are legible and unclipped.</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="H37" s="1" t="inlineStr">
         <is>
           <t>High / Artifact QA / visual check</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="I37" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="J37" s="1" t="inlineStr">
         <is>
           <t>Visual QA not established by XML/source inspection.</t>
         </is>
@@ -2473,47 +4044,47 @@
       <c r="A38" t="n">
         <v>37</v>
       </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Module 5 - Renter favorites, contact and inquiry</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="C38" s="1" t="inlineStr">
         <is>
           <t>M5-A4</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="1" t="inlineStr">
         <is>
           <t>SCRUM-127 AC4: trace to SCRUM-61/121 and ERD/RLS, and document assumptions/policy questions</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E38" s="1" t="inlineStr">
         <is>
           <t>Current Module 5 source docs, SCRUM-61/121 and ERD/RLS docs</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F38" s="1" t="inlineStr">
         <is>
           <t>1. Trace each module boundary and data/security element to its cited source. 2. Check no auth/map flow is duplicated. 3. Verify unresolved policy assumptions/questions are listed.</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="G38" s="1" t="inlineStr">
         <is>
           <t>Traceability is explicit; existing auth/map boundaries are reused; every unresolved policy question is visible and not treated as settled.</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="H38" s="1" t="inlineStr">
         <is>
           <t>High / Requirements trace / documentation</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="I38" s="1" t="inlineStr">
         <is>
           <t>NOT RUN</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="J38" s="1" t="inlineStr">
         <is>
           <t>Tests the planning artifact criterion, not application behavior.</t>
         </is>
@@ -2521,6 +4092,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:J38"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.3" right="0.3" top="0.35" bottom="0.35" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="5" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(SCRUM-165): reconcile module source coverage
</commit_message>
<xml_diff>
--- a/docs/testing/AbangCebu_Modules_3_4_5_Test_Cases.xlsx
+++ b/docs/testing/AbangCebu_Modules_3_4_5_Test_Cases.xlsx
@@ -12,9 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEST_CASES" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PRINT VIEW'!$A$4:$E$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PRINT VIEW'!$A$4:$E$45</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'PRINT VIEW'!$4:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'PRINT VIEW'!$A$1:$E$41</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'PRINT VIEW'!$A$1:$E$45</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'TEST DEFINITION'!$1:$2</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'TEST DEFINITION'!$A$1:$C$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'TEST_CASES'!$A$1:$J$38</definedName>
@@ -593,7 +593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1940,8 +1940,148 @@
         </is>
       </c>
     </row>
+    <row r="42" ht="280" customHeight="1">
+      <c r="A42" s="14" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>M3-08</t>
+        </is>
+      </c>
+      <c r="C42" s="14" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="D42" s="14" t="inlineStr">
+        <is>
+          <t>Critical / Security + authorization / role-policy gate
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E42" s="15" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-125 §4.1: authenticated landlord role required; SCRUM-121: deferred auth preserves safe intent; SCRUM-55/63: server-side role and ownership boundary
+PRECONDITIONS / SYNTHETIC DATA
+Disposable local DB; guest, authenticated renter, disabled/non-landlord, active landlord A; synthetic own and foreign property IDs; approved auth contract
+TEST STEPS
+1. As guest, attempt property create/edit and start the auth-gated listing action. 2. After test authentication, try again as renter and disabled/non-landlord. 3. As active landlord A, access own synthetic property. 4. As A, address landlord B record by known synthetic ID.
+EXPECTED RESULT
+Only an authenticated active landlord may perform permitted own-record operations. Guest intent follows the approved auth gate; other roles and foreign records fail closed without record-existence leakage or mutation.
+EVIDENCE / NOTES
+Synthetic identities/records only; assert server/database enforcement, not UI hiding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="350" customHeight="1">
+      <c r="A43" s="14" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>M3-09</t>
+        </is>
+      </c>
+      <c r="C43" s="14" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="D43" s="14" t="inlineStr">
+        <is>
+          <t>High / Lifecycle + negative / POLICY-SCHEMA GATE
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E43" s="15" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-125 §§2, 4.1, 4.2, 7: owner edits to approved listings and pause/archive transitions are policy/schema gated; unsupported mutations must not occur
+PRECONDITIONS / SYNTHETIC DATA
+Disposable local DB; landlord A owns a synthetic approved listing with a recorded version and availability; owner-approved edit/lifecycle contract, if available
+TEST STEPS
+1. Read the approved product/schema decision for edits to approved listings and supported archive/pause behavior. 2. If no explicit contract exists, attempt a bounded owner edit and unsupported pause/archive only in the disposable fixture. 3. Compare status, fields, version and audit data before/after. 4. If a contract exists, exercise only its permitted fields/transitions and denied alternatives.
+EXPECTED RESULT
+Without an approved contract, no edit/pause/archive success is reported and persisted state remains unchanged. With an approved contract, only its explicitly allowed owner edits/transitions succeed; unsupported transitions remain denied.
+EVIDENCE / NOTES
+No approved contract means no mutation. Do not infer archive as pause/unpublish.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="350" customHeight="1">
+      <c r="A44" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>M4-07</t>
+        </is>
+      </c>
+      <c r="C44" s="14" t="inlineStr">
+        <is>
+          <t>M4 — Admin moderation</t>
+        </is>
+      </c>
+      <c r="D44" s="14" t="inlineStr">
+        <is>
+          <t>Critical / Security + policy boundary / KYC evidence gate
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E44" s="15" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-126 §§3, 5, 7: insufficient/suspicious KYC evidence is not approval; escalation and correction are blocked absent approved authority/owner flow
+PRECONDITIONS / SYNTHETIC DATA
+Disposable local DB; active admin and synthetic KYC submission using placeholder metadata only; insufficient/suspicious evidence fixture; no real ID image or personal data
+TEST STEPS
+1. Review a synthetic submission with missing, unreadable, or inconsistent evidence. 2. Attempt verification. 3. Inspect supported correction, escalation and audit gates. 4. Attempt an escalation only if a fixture exposes one and record whether an approved policy authorizes it. 5. Check status and sensitive-data exposure.
+EXPECTED RESULT
+Insufficient/suspicious evidence is never verified by default. Without an approved correction/escalation policy, the supported state remains unchanged; no unsupported intake, escalation, suspension or new status is created. No KYC bytes or storage path is exposed.
+EVIDENCE / NOTES
+Use placeholder metadata only; correction/escalation require explicit policy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="280" customHeight="1">
+      <c r="A45" s="14" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>M5-08</t>
+        </is>
+      </c>
+      <c r="C45" s="14" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="D45" s="14" t="inlineStr">
+        <is>
+          <t>Critical / Security + redirect/privacy / tamper-resistance gate
+STATUS: NOT RUN</t>
+        </is>
+      </c>
+      <c r="E45" s="15" t="inlineStr">
+        <is>
+          <t>REQUIREMENT / CRITERION TRACE
+SCRUM-127 AC2; SCRUM-121: restore the same listing and action through a bounded same-origin intent; reject tampered target/action and unsafe redirects
+PRECONDITIONS / SYNTHETIC DATA
+Isolated auth test; guest action on synthetic listing A; safe same-origin return path; synthetic renter; no credentials stored in the intent
+TEST STEPS
+1. Start a favorite/contact/inquiry intent for listing A as guest. 2. Tamper the return target to an external origin, protocol-relative URL, or javascript: URL. 3. Change the stored listing ID or action before auth completion. 4. Replay the intent for a different listing after authentication. 5. Compare resulting writes and contact response.
+EXPECTED RESULT
+Only the original allowlisted same-origin route, listing A, and exact action may resume after renter authorization. Invalid, changed, or replayed intent is rejected without a favorite/inquiry mutation, open redirect, or contact disclosure.
+EVIDENCE / NOTES
+Design-level case; never store credentials or sensitive form data in pending intent.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:E41"/>
+  <autoFilter ref="A4:E45"/>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
@@ -1956,7 +2096,7 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <rowBreaks count="18" manualBreakCount="18">
+  <rowBreaks count="20" manualBreakCount="20">
     <brk id="6" min="0" max="16383" man="1"/>
     <brk id="8" min="0" max="16383" man="1"/>
     <brk id="10" min="0" max="16383" man="1"/>
@@ -1975,6 +2115,8 @@
     <brk id="36" min="0" max="16383" man="1"/>
     <brk id="38" min="0" max="16383" man="1"/>
     <brk id="40" min="0" max="16383" man="1"/>
+    <brk id="42" min="0" max="16383" man="1"/>
+    <brk id="44" min="0" max="16383" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
@@ -1985,7 +2127,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr autoPageBreaks="0" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2049,7 +2191,7 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>Traceable functional, security, integration, and recovery test cases. Each of the four acceptance criteria in the live Jira descriptions for SCRUM-125/126/127 maps to one or more proposed case IDs. Original binary source attachments and referenced Module 3-5 spec files were not content-reviewed, so full source-spec coverage remains unverified. Resolve listed product/schema gates before execution; this workbook does not assert product behavior or execution.</t>
+          <t>Planning-only specification: 41 proposed cases; all remain NOT RUN. The 12 live Jira acceptance criteria map to case IDs in the plan. Module 3–5 repository specs and Draw.io sources were reconciled against the exact commit snapshots and hashes listed in the plan. Original Jira source attachment bytes were not retrievable for binary comparison; this does not establish product, runtime, staging, or production behavior.</t>
         </is>
       </c>
     </row>
@@ -2158,6 +2300,54 @@
       <c r="B14" s="1" t="inlineStr">
         <is>
           <t>None. Results and actual executor/date must be recorded by the authorized QA session when executed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>Module 3 source snapshot</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>SCRUM-125 specs/flowcharts: 896abf636d8dba0818da23728953eca4505a22e7; see plan for per-file SHA-256.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>Module 4 source snapshot</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>SCRUM-126 spec/flowcharts: f3fb5841578831979327a66f95cecad6aabad6d7; see plan for per-file SHA-256.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="36" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>Module 5 source snapshot</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>SCRUM-127 spec/flowcharts: 507436d603ddb904d0a6ffe84cfaf74a4c973a4c; see plan for per-file SHA-256.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="36" customHeight="1">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>Source boundary</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>Original Jira source attachment binaries were not retrieved or hash-compared. Product tests remain NOT RUN.</t>
         </is>
       </c>
     </row>
@@ -2173,7 +2363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4090,6 +4280,206 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>M3-08</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>SCRUM-125 §4.1: authenticated landlord role required; SCRUM-121: deferred auth preserves safe intent; SCRUM-55/63: server-side role and ownership boundary</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Disposable local DB; guest, authenticated renter, disabled/non-landlord, active landlord A; synthetic own and foreign property IDs; approved auth contract</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>1. As guest, attempt property create/edit and start the auth-gated listing action. 2. After test authentication, try again as renter and disabled/non-landlord. 3. As active landlord A, access own synthetic property. 4. As A, address landlord B record by known synthetic ID.</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Only an authenticated active landlord may perform permitted own-record operations. Guest intent follows the approved auth gate; other roles and foreign records fail closed without record-existence leakage or mutation.</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Critical / Security + authorization / role-policy gate</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Synthetic identities/records only; assert server/database enforcement, not UI hiding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>M3 — Landlord listings</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>M3-09</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>SCRUM-125 §§2, 4.1, 4.2, 7: owner edits to approved listings and pause/archive transitions are policy/schema gated; unsupported mutations must not occur</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Disposable local DB; landlord A owns a synthetic approved listing with a recorded version and availability; owner-approved edit/lifecycle contract, if available</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>1. Read the approved product/schema decision for edits to approved listings and supported archive/pause behavior. 2. If no explicit contract exists, attempt a bounded owner edit and unsupported pause/archive only in the disposable fixture. 3. Compare status, fields, version and audit data before/after. 4. If a contract exists, exercise only its permitted fields/transitions and denied alternatives.</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Without an approved contract, no edit/pause/archive success is reported and persisted state remains unchanged. With an approved contract, only its explicitly allowed owner edits/transitions succeed; unsupported transitions remain denied.</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>High / Lifecycle + negative / POLICY-SCHEMA GATE</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>No approved contract means no mutation. Do not infer archive as pause/unpublish.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>M4 — Admin moderation</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>M4-07</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>SCRUM-126 §§3, 5, 7: insufficient/suspicious KYC evidence is not approval; escalation and correction are blocked absent approved authority/owner flow</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Disposable local DB; active admin and synthetic KYC submission using placeholder metadata only; insufficient/suspicious evidence fixture; no real ID image or personal data</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>1. Review a synthetic submission with missing, unreadable, or inconsistent evidence. 2. Attempt verification. 3. Inspect supported correction, escalation and audit gates. 4. Attempt an escalation only if a fixture exposes one and record whether an approved policy authorizes it. 5. Check status and sensitive-data exposure.</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Insufficient/suspicious evidence is never verified by default. Without an approved correction/escalation policy, the supported state remains unchanged; no unsupported intake, escalation, suspension or new status is created. No KYC bytes or storage path is exposed.</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Critical / Security + policy boundary / KYC evidence gate</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Use placeholder metadata only; correction/escalation require explicit policy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>M5 — Renter engagement</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>M5-08</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>SCRUM-127 AC2; SCRUM-121: restore the same listing and action through a bounded same-origin intent; reject tampered target/action and unsafe redirects</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Isolated auth test; guest action on synthetic listing A; safe same-origin return path; synthetic renter; no credentials stored in the intent</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>1. Start a favorite/contact/inquiry intent for listing A as guest. 2. Tamper the return target to an external origin, protocol-relative URL, or javascript: URL. 3. Change the stored listing ID or action before auth completion. 4. Replay the intent for a different listing after authentication. 5. Compare resulting writes and contact response.</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Only the original allowlisted same-origin route, listing A, and exact action may resume after renter authorization. Invalid, changed, or replayed intent is rejected without a favorite/inquiry mutation, open redirect, or contact disclosure.</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Critical / Security + redirect/privacy / tamper-resistance gate</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>NOT RUN</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Design-level case; never store credentials or sensitive form data in pending intent.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J38"/>
   <pageMargins left="0.3" right="0.3" top="0.35" bottom="0.35" header="0.5" footer="0.5"/>

</xml_diff>